<commit_message>
Add terminology intelligence platform initial structure
</commit_message>
<xml_diff>
--- a/tools/manufacturing-terminology-intelligence-platform/glossary.xlsx
+++ b/tools/manufacturing-terminology-intelligence-platform/glossary.xlsx
@@ -407,4 +407,10 @@
     <oddHeader>&amp;L&amp;"Meiyo"&amp;10&amp;K000000 •• PROTECTED 関係者外秘&amp;1#_x000D_</oddHeader>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{fbb3c382-541a-4789-80ed-24b21ea5b276}" enabled="1" method="Standard" siteId="{8c642d1d-d709-47b0-ab10-080af10798fb}" contentBits="1" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>